<commit_message>
làm bài tập section 1 phần tính từ, trạng từ
</commit_message>
<xml_diff>
--- a/Khóa toeic prep/0-300/Ngữ pháp/lý thuyết/Ngữ pháp.xlsx
+++ b/Khóa toeic prep/0-300/Ngữ pháp/lý thuyết/Ngữ pháp.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\toeic learning\Khóa toeic prep\0-300\Ngữ pháp\lý thuyết\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\toeic\0-300\Khóa toeic prep\0-300\Ngữ pháp\lý thuyết\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A35B03F-E718-4CA3-9FAA-E27BB5AEA4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E88CBC-2285-491C-AC7E-B43271A9C610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38265" yWindow="4545" windowWidth="15675" windowHeight="10935" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Danh từ" sheetId="2" r:id="rId1"/>
     <sheet name="2. Động từ" sheetId="5" r:id="rId2"/>
     <sheet name="3. Đại từ" sheetId="4" r:id="rId3"/>
-    <sheet name="Template (2)" sheetId="6" r:id="rId4"/>
+    <sheet name="4. Tính từ &amp; Trạng từ" sheetId="7" r:id="rId4"/>
+    <sheet name="Template (2)" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="371">
   <si>
     <t>Người</t>
   </si>
@@ -1799,6 +1800,159 @@
   </si>
   <si>
     <t>By + đại từ phản thân: tự làm 1 mình không có sự giúp đỡ của người khác</t>
+  </si>
+  <si>
+    <t>1 Tính từ</t>
+  </si>
+  <si>
+    <t>good-looking: ưa nhìn</t>
+  </si>
+  <si>
+    <t>modern: hiện đại</t>
+  </si>
+  <si>
+    <t>fun: thú vị</t>
+  </si>
+  <si>
+    <t>healthy: khỏe mạnh</t>
+  </si>
+  <si>
+    <t>fashionable: thời trang</t>
+  </si>
+  <si>
+    <t>VD:</t>
+  </si>
+  <si>
+    <t>1.1 Khái niệm: Tính từ là từ mô tả đặc điểm tính chất của 1 người, vật , hay sự việc nào đó</t>
+  </si>
+  <si>
+    <t>1.2 Vị trí</t>
+  </si>
+  <si>
+    <t>TÍnh từ có thể đứng trước danh từ</t>
+  </si>
+  <si>
+    <t>tính từ có thể đứng sau động từ</t>
+  </si>
+  <si>
+    <t>+ tính từ thường hay theo sau động từ tobe</t>
+  </si>
+  <si>
+    <t>it is cold outside( ở ngoài trời đang lạnh.)</t>
+  </si>
+  <si>
+    <t>+ theo sau các động từ sau: seem, look, become, get, feel, sound, taste, smell, appear</t>
+  </si>
+  <si>
+    <t>Loại tính từ</t>
+  </si>
+  <si>
+    <t>Trường hợp chỉ đi sau To be/Verb</t>
+  </si>
+  <si>
+    <t>Trường hợp thay thế (đứng trước Noun)</t>
+  </si>
+  <si>
+    <t>Ghi chú nhanh</t>
+  </si>
+  <si>
+    <t>Nhóm bắt đầu bằng 'a-'</t>
+  </si>
+  <si>
+    <t>Afraid, Asleep, Alive, Alike, Alone, Awake</t>
+  </si>
+  <si>
+    <t>Frightened, Sleeping, Live, Similar</t>
+  </si>
+  <si>
+    <t>Tuyệt đối không đặt 'a-' trước danh từ.</t>
+  </si>
+  <si>
+    <t>Sức khỏe &amp; Cảm xúc</t>
+  </si>
+  <si>
+    <t>Ill, Well, Glad, Content</t>
+  </si>
+  <si>
+    <t>Sick, Healthy, Happy</t>
+  </si>
+  <si>
+    <t>Dùng 'He is ill' nhưng phải là 'A sick man'.</t>
+  </si>
+  <si>
+    <t>Tóm tắt</t>
+  </si>
+  <si>
+    <t>Chỉ làm vị ngữ (Predicative only)</t>
+  </si>
+  <si>
+    <t>Tính từ định ngữ tương đương</t>
+  </si>
+  <si>
+    <t>Dùng khi mô tả trạng thái tạm thời.</t>
+  </si>
+  <si>
+    <t>1.3 trường hợp đặc biệt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Các loại tính từ </t>
+  </si>
+  <si>
+    <t>2.1 các loại tính từ</t>
+  </si>
+  <si>
+    <t>+ Shape: hình dạng</t>
+  </si>
+  <si>
+    <t>+ purpose: mục đích</t>
+  </si>
+  <si>
+    <t>+ material: chất liệu</t>
+  </si>
+  <si>
+    <t>+ size: kích thước</t>
+  </si>
+  <si>
+    <t>+ origin: nguồn gốc</t>
+  </si>
+  <si>
+    <t>+ age: tuổi tác</t>
+  </si>
+  <si>
+    <t>+ opinion: ý kiến</t>
+  </si>
+  <si>
+    <t>VD: cone: hình côn</t>
+  </si>
+  <si>
+    <t>VD: old: già</t>
+  </si>
+  <si>
+    <t>+ color: màu sắc</t>
+  </si>
+  <si>
+    <t>VD: wild: hoang dã</t>
+  </si>
+  <si>
+    <t>VD: brown</t>
+  </si>
+  <si>
+    <t>VD: cleaning: như một công cụ lau chùi</t>
+  </si>
+  <si>
+    <t>2.2 thứ tự của tính từ</t>
+  </si>
+  <si>
+    <t>Opinion -&gt; Size -&gt; Age -&gt; Shape -&gt; Color -&gt; Origin -&gt; Material -&gt; Purpose</t>
+  </si>
+  <si>
+    <t>VD:  strange: lạ, happy: bvui</t>
+  </si>
+  <si>
+    <t>VD: large: rộng, big…</t>
+  </si>
+  <si>
+    <t>VD: wooden: gỗ , brick: gach…</t>
   </si>
 </sst>
 </file>
@@ -1830,12 +1984,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="10">
@@ -1945,7 +2105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1979,6 +2139,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2001,9 +2173,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2403,364 +2572,364 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4F4B3F8-BF9C-43F8-86EE-68B07098D7B4}">
   <dimension ref="A1:O155"/>
-  <sheetFormatPr defaultColWidth="2.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27" s="6"/>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29" s="5"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31" s="6"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="5"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="6"/>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="5"/>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="6"/>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="5"/>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="6"/>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="5"/>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="6"/>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="5"/>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="6"/>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="5"/>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="6"/>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="5"/>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="6"/>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="5"/>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="6"/>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="97" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="99" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B99" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="101" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="102" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C102" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="103" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C103" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="105" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C105" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="107" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="108" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C108" t="s">
         <v>58</v>
       </c>
@@ -2768,7 +2937,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="109" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C109" t="s">
         <v>60</v>
       </c>
@@ -2776,258 +2945,258 @@
         <v>61</v>
       </c>
     </row>
-    <row r="111" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="112" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="114" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="116" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="118" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="120" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B120" s="13" t="s">
+    <row r="120" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B120" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="C120" s="13"/>
-      <c r="D120" s="13"/>
-      <c r="E120" s="13"/>
-      <c r="F120" s="13"/>
-      <c r="G120" s="13"/>
-      <c r="H120" s="13" t="s">
+      <c r="C120" s="17"/>
+      <c r="D120" s="17"/>
+      <c r="E120" s="17"/>
+      <c r="F120" s="17"/>
+      <c r="G120" s="17"/>
+      <c r="H120" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="I120" s="13"/>
-      <c r="J120" s="13"/>
-      <c r="K120" s="13"/>
-      <c r="L120" s="13"/>
-      <c r="M120" s="13"/>
-    </row>
-    <row r="121" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B121" s="13" t="s">
+      <c r="I120" s="17"/>
+      <c r="J120" s="17"/>
+      <c r="K120" s="17"/>
+      <c r="L120" s="17"/>
+      <c r="M120" s="17"/>
+    </row>
+    <row r="121" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B121" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C121" s="13"/>
-      <c r="D121" s="13"/>
-      <c r="E121" s="13"/>
-      <c r="F121" s="13"/>
-      <c r="G121" s="13"/>
-      <c r="H121" s="13" t="s">
+      <c r="C121" s="17"/>
+      <c r="D121" s="17"/>
+      <c r="E121" s="17"/>
+      <c r="F121" s="17"/>
+      <c r="G121" s="17"/>
+      <c r="H121" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="I121" s="13"/>
-      <c r="J121" s="13"/>
-      <c r="K121" s="13"/>
-      <c r="L121" s="13"/>
-      <c r="M121" s="13"/>
-    </row>
-    <row r="122" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B122" s="13" t="s">
+      <c r="I121" s="17"/>
+      <c r="J121" s="17"/>
+      <c r="K121" s="17"/>
+      <c r="L121" s="17"/>
+      <c r="M121" s="17"/>
+    </row>
+    <row r="122" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B122" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="C122" s="13"/>
-      <c r="D122" s="13"/>
-      <c r="E122" s="13"/>
-      <c r="F122" s="13"/>
-      <c r="G122" s="13"/>
-      <c r="H122" s="13" t="s">
+      <c r="C122" s="17"/>
+      <c r="D122" s="17"/>
+      <c r="E122" s="17"/>
+      <c r="F122" s="17"/>
+      <c r="G122" s="17"/>
+      <c r="H122" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="I122" s="13"/>
-      <c r="J122" s="13"/>
-      <c r="K122" s="13"/>
-      <c r="L122" s="13"/>
-      <c r="M122" s="13"/>
-    </row>
-    <row r="123" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B123" s="13" t="s">
+      <c r="I122" s="17"/>
+      <c r="J122" s="17"/>
+      <c r="K122" s="17"/>
+      <c r="L122" s="17"/>
+      <c r="M122" s="17"/>
+    </row>
+    <row r="123" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B123" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="C123" s="13"/>
-      <c r="D123" s="13"/>
-      <c r="E123" s="13"/>
-      <c r="F123" s="13"/>
-      <c r="G123" s="13"/>
-      <c r="H123" s="13" t="s">
+      <c r="C123" s="17"/>
+      <c r="D123" s="17"/>
+      <c r="E123" s="17"/>
+      <c r="F123" s="17"/>
+      <c r="G123" s="17"/>
+      <c r="H123" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="I123" s="13"/>
-      <c r="J123" s="13"/>
-      <c r="K123" s="13"/>
-      <c r="L123" s="13"/>
-      <c r="M123" s="13"/>
-    </row>
-    <row r="124" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B124" s="13" t="s">
+      <c r="I123" s="17"/>
+      <c r="J123" s="17"/>
+      <c r="K123" s="17"/>
+      <c r="L123" s="17"/>
+      <c r="M123" s="17"/>
+    </row>
+    <row r="124" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B124" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C124" s="13"/>
-      <c r="D124" s="13"/>
-      <c r="E124" s="13"/>
-      <c r="F124" s="13"/>
-      <c r="G124" s="13"/>
-      <c r="H124" s="13" t="s">
+      <c r="C124" s="17"/>
+      <c r="D124" s="17"/>
+      <c r="E124" s="17"/>
+      <c r="F124" s="17"/>
+      <c r="G124" s="17"/>
+      <c r="H124" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="I124" s="13"/>
-      <c r="J124" s="13"/>
-      <c r="K124" s="13"/>
-      <c r="L124" s="13"/>
-      <c r="M124" s="13"/>
-    </row>
-    <row r="125" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B125" s="13" t="s">
+      <c r="I124" s="17"/>
+      <c r="J124" s="17"/>
+      <c r="K124" s="17"/>
+      <c r="L124" s="17"/>
+      <c r="M124" s="17"/>
+    </row>
+    <row r="125" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B125" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="C125" s="13"/>
-      <c r="D125" s="13"/>
-      <c r="E125" s="13"/>
-      <c r="F125" s="13"/>
-      <c r="G125" s="13"/>
-      <c r="H125" s="13" t="s">
+      <c r="C125" s="17"/>
+      <c r="D125" s="17"/>
+      <c r="E125" s="17"/>
+      <c r="F125" s="17"/>
+      <c r="G125" s="17"/>
+      <c r="H125" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="I125" s="13"/>
-      <c r="J125" s="13"/>
-      <c r="K125" s="13"/>
-      <c r="L125" s="13"/>
-      <c r="M125" s="13"/>
-    </row>
-    <row r="126" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B126" s="13" t="s">
+      <c r="I125" s="17"/>
+      <c r="J125" s="17"/>
+      <c r="K125" s="17"/>
+      <c r="L125" s="17"/>
+      <c r="M125" s="17"/>
+    </row>
+    <row r="126" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B126" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="C126" s="13"/>
-      <c r="D126" s="13"/>
-      <c r="E126" s="13"/>
-      <c r="F126" s="13"/>
-      <c r="G126" s="13"/>
-      <c r="H126" s="13" t="s">
+      <c r="C126" s="17"/>
+      <c r="D126" s="17"/>
+      <c r="E126" s="17"/>
+      <c r="F126" s="17"/>
+      <c r="G126" s="17"/>
+      <c r="H126" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="I126" s="13"/>
-      <c r="J126" s="13"/>
-      <c r="K126" s="13"/>
-      <c r="L126" s="13"/>
-      <c r="M126" s="13"/>
-    </row>
-    <row r="127" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B127" s="13" t="s">
+      <c r="I126" s="17"/>
+      <c r="J126" s="17"/>
+      <c r="K126" s="17"/>
+      <c r="L126" s="17"/>
+      <c r="M126" s="17"/>
+    </row>
+    <row r="127" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B127" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C127" s="13"/>
-      <c r="D127" s="13"/>
-      <c r="E127" s="13"/>
-      <c r="F127" s="13"/>
-      <c r="G127" s="13"/>
-      <c r="H127" s="13" t="s">
+      <c r="C127" s="17"/>
+      <c r="D127" s="17"/>
+      <c r="E127" s="17"/>
+      <c r="F127" s="17"/>
+      <c r="G127" s="17"/>
+      <c r="H127" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="I127" s="13"/>
-      <c r="J127" s="13"/>
-      <c r="K127" s="13"/>
-      <c r="L127" s="13"/>
-      <c r="M127" s="13"/>
-    </row>
-    <row r="128" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B128" s="13" t="s">
+      <c r="I127" s="17"/>
+      <c r="J127" s="17"/>
+      <c r="K127" s="17"/>
+      <c r="L127" s="17"/>
+      <c r="M127" s="17"/>
+    </row>
+    <row r="128" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B128" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="C128" s="13"/>
-      <c r="D128" s="13"/>
-      <c r="E128" s="13"/>
-      <c r="F128" s="13"/>
-      <c r="G128" s="13"/>
-      <c r="H128" s="13" t="s">
+      <c r="C128" s="17"/>
+      <c r="D128" s="17"/>
+      <c r="E128" s="17"/>
+      <c r="F128" s="17"/>
+      <c r="G128" s="17"/>
+      <c r="H128" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I128" s="13"/>
-      <c r="J128" s="13"/>
-      <c r="K128" s="13"/>
-      <c r="L128" s="13"/>
-      <c r="M128" s="13"/>
-    </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B129" s="13"/>
-      <c r="C129" s="13"/>
-      <c r="D129" s="13"/>
-      <c r="E129" s="13"/>
-      <c r="F129" s="13"/>
-      <c r="G129" s="13"/>
-      <c r="H129" s="13"/>
-      <c r="I129" s="13"/>
-      <c r="J129" s="13"/>
-      <c r="K129" s="13"/>
-      <c r="L129" s="13"/>
-      <c r="M129" s="13"/>
-    </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="I128" s="17"/>
+      <c r="J128" s="17"/>
+      <c r="K128" s="17"/>
+      <c r="L128" s="17"/>
+      <c r="M128" s="17"/>
+    </row>
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B129" s="17"/>
+      <c r="C129" s="17"/>
+      <c r="D129" s="17"/>
+      <c r="E129" s="17"/>
+      <c r="F129" s="17"/>
+      <c r="G129" s="17"/>
+      <c r="H129" s="17"/>
+      <c r="I129" s="17"/>
+      <c r="J129" s="17"/>
+      <c r="K129" s="17"/>
+      <c r="L129" s="17"/>
+      <c r="M129" s="17"/>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B140" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="145" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="145" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>95</v>
       </c>
@@ -3035,12 +3204,12 @@
         <v>96</v>
       </c>
     </row>
-    <row r="146" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="146" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="147" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="147" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
         <v>98</v>
       </c>
@@ -3054,12 +3223,12 @@
         <v>101</v>
       </c>
     </row>
-    <row r="149" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="151" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="151" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
         <v>102</v>
       </c>
@@ -3070,7 +3239,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="153" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="153" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
         <v>103</v>
       </c>
@@ -3081,7 +3250,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="155" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="155" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B155" t="s">
         <v>107</v>
       </c>
@@ -3117,289 +3286,289 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F6D20B-34C8-444A-B778-F16F19BF2F96}">
   <dimension ref="A1:T193"/>
-  <sheetFormatPr defaultColWidth="2.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="2.81640625" customWidth="1"/>
+    <col min="2" max="2" width="2.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C4" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="7" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C10" s="7" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C11" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C12" s="7" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C13" s="7" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C14" s="7" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C18" s="7" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="21" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B24" s="7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B25" s="7" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B26" s="7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B27" s="7"/>
       <c r="C27" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28" s="7"/>
       <c r="C28" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B29" s="7"/>
       <c r="C29" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B30" s="7"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32" s="7" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C33" s="7" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C34" s="7" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C35" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="9" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="9" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40" s="3"/>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="10" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42" s="2"/>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43" s="6"/>
       <c r="C43" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44" s="3"/>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45" s="5"/>
       <c r="C45" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" s="2"/>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47" s="10" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48" s="3"/>
       <c r="C48" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B49" s="5"/>
       <c r="C49" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B50" s="2"/>
       <c r="C50" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B51" s="6"/>
       <c r="C51" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B52" s="3"/>
     </row>
-    <row r="53" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B54" s="4"/>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B55" s="10" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B56" s="10" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B57" s="11" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B58" s="5"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B59" s="10" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B61" s="3"/>
       <c r="C61" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B62" s="5"/>
       <c r="C62" s="7" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B63" s="2"/>
       <c r="C63" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B64" s="6" t="s">
         <v>156</v>
       </c>
@@ -3407,626 +3576,626 @@
         <v>157</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65" s="3"/>
       <c r="C65" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="3"/>
       <c r="C66" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67" s="5"/>
       <c r="C67" s="7" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68" s="2"/>
       <c r="C68" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69" s="6"/>
       <c r="C69" s="7" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70" s="3"/>
       <c r="C70" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C71" s="7" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72" s="4"/>
       <c r="C72" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73" s="5"/>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74" s="10" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75" s="6"/>
       <c r="C75" s="7" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76" s="3"/>
       <c r="C76" s="7" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77" s="5"/>
       <c r="C77" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B78" s="2"/>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B79" s="10" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B80" s="3"/>
       <c r="C80" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C83" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="B93" s="16" t="s">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B93" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="C93" s="16"/>
-      <c r="D93" s="16"/>
-      <c r="E93" s="16"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="16"/>
-      <c r="H93" s="16" t="s">
+      <c r="C93" s="20"/>
+      <c r="D93" s="20"/>
+      <c r="E93" s="20"/>
+      <c r="F93" s="20"/>
+      <c r="G93" s="20"/>
+      <c r="H93" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="I93" s="16"/>
-      <c r="J93" s="16"/>
-      <c r="K93" s="16"/>
-      <c r="L93" s="16"/>
-      <c r="M93" s="16"/>
-    </row>
-    <row r="94" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B94" s="14" t="s">
+      <c r="I93" s="20"/>
+      <c r="J93" s="20"/>
+      <c r="K93" s="20"/>
+      <c r="L93" s="20"/>
+      <c r="M93" s="20"/>
+    </row>
+    <row r="94" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="C94" s="14"/>
-      <c r="D94" s="14"/>
-      <c r="E94" s="14"/>
-      <c r="F94" s="14"/>
-      <c r="G94" s="14"/>
-      <c r="H94" s="15" t="s">
+      <c r="C94" s="18"/>
+      <c r="D94" s="18"/>
+      <c r="E94" s="18"/>
+      <c r="F94" s="18"/>
+      <c r="G94" s="18"/>
+      <c r="H94" s="19" t="s">
         <v>182</v>
       </c>
-      <c r="I94" s="15"/>
-      <c r="J94" s="15"/>
-      <c r="K94" s="15"/>
-      <c r="L94" s="15"/>
-      <c r="M94" s="15"/>
-    </row>
-    <row r="95" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B95" s="14" t="s">
+      <c r="I94" s="19"/>
+      <c r="J94" s="19"/>
+      <c r="K94" s="19"/>
+      <c r="L94" s="19"/>
+      <c r="M94" s="19"/>
+    </row>
+    <row r="95" spans="1:13" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B95" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C95" s="14"/>
-      <c r="D95" s="14"/>
-      <c r="E95" s="14"/>
-      <c r="F95" s="14"/>
-      <c r="G95" s="14"/>
-      <c r="H95" s="15" t="s">
+      <c r="C95" s="18"/>
+      <c r="D95" s="18"/>
+      <c r="E95" s="18"/>
+      <c r="F95" s="18"/>
+      <c r="G95" s="18"/>
+      <c r="H95" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="I95" s="15"/>
-      <c r="J95" s="15"/>
-      <c r="K95" s="15"/>
-      <c r="L95" s="15"/>
-      <c r="M95" s="15"/>
-    </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="I95" s="19"/>
+      <c r="J95" s="19"/>
+      <c r="K95" s="19"/>
+      <c r="L95" s="19"/>
+      <c r="M95" s="19"/>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="7"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B119" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C120" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C121" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C122" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D123" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D124" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C126" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C127" s="7" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C128" s="7" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="129" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="129" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C129" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="131" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="133" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C133" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="135" spans="2:20" x14ac:dyDescent="0.35">
-      <c r="C135" s="15" t="s">
+    <row r="135" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C135" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="D135" s="15"/>
-      <c r="E135" s="15"/>
-      <c r="F135" s="15"/>
-      <c r="G135" s="15"/>
-      <c r="H135" s="15"/>
-      <c r="I135" s="15" t="s">
+      <c r="D135" s="19"/>
+      <c r="E135" s="19"/>
+      <c r="F135" s="19"/>
+      <c r="G135" s="19"/>
+      <c r="H135" s="19"/>
+      <c r="I135" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="J135" s="15"/>
-      <c r="K135" s="15"/>
-      <c r="L135" s="15"/>
-      <c r="M135" s="15"/>
-      <c r="N135" s="15"/>
-      <c r="O135" s="17" t="s">
+      <c r="J135" s="19"/>
+      <c r="K135" s="19"/>
+      <c r="L135" s="19"/>
+      <c r="M135" s="19"/>
+      <c r="N135" s="19"/>
+      <c r="O135" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="P135" s="18"/>
-      <c r="Q135" s="18"/>
-      <c r="R135" s="18"/>
-      <c r="S135" s="18"/>
-      <c r="T135" s="19"/>
-    </row>
-    <row r="136" spans="2:20" x14ac:dyDescent="0.35">
-      <c r="C136" s="15" t="s">
+      <c r="P135" s="22"/>
+      <c r="Q135" s="22"/>
+      <c r="R135" s="22"/>
+      <c r="S135" s="22"/>
+      <c r="T135" s="23"/>
+    </row>
+    <row r="136" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C136" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="D136" s="15"/>
-      <c r="E136" s="15"/>
-      <c r="F136" s="15"/>
-      <c r="G136" s="15"/>
-      <c r="H136" s="15"/>
-      <c r="I136" s="15" t="s">
+      <c r="D136" s="19"/>
+      <c r="E136" s="19"/>
+      <c r="F136" s="19"/>
+      <c r="G136" s="19"/>
+      <c r="H136" s="19"/>
+      <c r="I136" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="J136" s="15"/>
-      <c r="K136" s="15"/>
-      <c r="L136" s="15"/>
-      <c r="M136" s="15"/>
-      <c r="N136" s="15"/>
-      <c r="O136" s="20"/>
-      <c r="P136" s="21"/>
-      <c r="Q136" s="21"/>
-      <c r="R136" s="21"/>
-      <c r="S136" s="21"/>
-      <c r="T136" s="22"/>
-    </row>
-    <row r="137" spans="2:20" x14ac:dyDescent="0.35">
-      <c r="C137" s="15" t="s">
+      <c r="J136" s="19"/>
+      <c r="K136" s="19"/>
+      <c r="L136" s="19"/>
+      <c r="M136" s="19"/>
+      <c r="N136" s="19"/>
+      <c r="O136" s="24"/>
+      <c r="P136" s="16"/>
+      <c r="Q136" s="16"/>
+      <c r="R136" s="16"/>
+      <c r="S136" s="16"/>
+      <c r="T136" s="25"/>
+    </row>
+    <row r="137" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C137" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="D137" s="15"/>
-      <c r="E137" s="15"/>
-      <c r="F137" s="15"/>
-      <c r="G137" s="15"/>
-      <c r="H137" s="15"/>
-      <c r="I137" s="15" t="s">
+      <c r="D137" s="19"/>
+      <c r="E137" s="19"/>
+      <c r="F137" s="19"/>
+      <c r="G137" s="19"/>
+      <c r="H137" s="19"/>
+      <c r="I137" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="J137" s="15"/>
-      <c r="K137" s="15"/>
-      <c r="L137" s="15"/>
-      <c r="M137" s="15"/>
-      <c r="N137" s="15"/>
-      <c r="O137" s="20"/>
-      <c r="P137" s="21"/>
-      <c r="Q137" s="21"/>
-      <c r="R137" s="21"/>
-      <c r="S137" s="21"/>
-      <c r="T137" s="22"/>
-    </row>
-    <row r="138" spans="2:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C138" s="14" t="s">
+      <c r="J137" s="19"/>
+      <c r="K137" s="19"/>
+      <c r="L137" s="19"/>
+      <c r="M137" s="19"/>
+      <c r="N137" s="19"/>
+      <c r="O137" s="24"/>
+      <c r="P137" s="16"/>
+      <c r="Q137" s="16"/>
+      <c r="R137" s="16"/>
+      <c r="S137" s="16"/>
+      <c r="T137" s="25"/>
+    </row>
+    <row r="138" spans="2:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C138" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="D138" s="14"/>
-      <c r="E138" s="14"/>
-      <c r="F138" s="14"/>
-      <c r="G138" s="14"/>
-      <c r="H138" s="14"/>
-      <c r="I138" s="15" t="s">
+      <c r="D138" s="18"/>
+      <c r="E138" s="18"/>
+      <c r="F138" s="18"/>
+      <c r="G138" s="18"/>
+      <c r="H138" s="18"/>
+      <c r="I138" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="J138" s="15"/>
-      <c r="K138" s="15"/>
-      <c r="L138" s="15"/>
-      <c r="M138" s="15"/>
-      <c r="N138" s="15"/>
-      <c r="O138" s="23"/>
-      <c r="P138" s="24"/>
-      <c r="Q138" s="24"/>
-      <c r="R138" s="24"/>
-      <c r="S138" s="24"/>
-      <c r="T138" s="25"/>
-    </row>
-    <row r="140" spans="2:20" x14ac:dyDescent="0.35">
+      <c r="J138" s="19"/>
+      <c r="K138" s="19"/>
+      <c r="L138" s="19"/>
+      <c r="M138" s="19"/>
+      <c r="N138" s="19"/>
+      <c r="O138" s="26"/>
+      <c r="P138" s="27"/>
+      <c r="Q138" s="27"/>
+      <c r="R138" s="27"/>
+      <c r="S138" s="27"/>
+      <c r="T138" s="28"/>
+    </row>
+    <row r="140" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C140" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="142" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="142" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C142" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="143" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="143" spans="2:20" x14ac:dyDescent="0.25">
       <c r="D143" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="144" spans="2:20" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:20" x14ac:dyDescent="0.25">
       <c r="D144" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C146" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B150" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C151" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C152" s="7" t="s">
         <v>228</v>
       </c>
       <c r="M152" s="7"/>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C153" s="7" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C154" s="7" t="s">
         <v>230</v>
       </c>
       <c r="M154" s="7"/>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C155" s="7" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C156" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B157" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C159" s="7" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C160" s="7" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="162" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="162" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C162" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="163" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="163" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C163" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="164" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C164" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="165" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="165" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C165" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="166" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C166" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="168" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B168" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="169" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C169" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="170" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="170" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D170" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="171" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D171" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="172" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D172" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="173" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D173" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="174" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D174" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="175" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D175" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="176" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C176" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="178" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="178" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B178" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="180" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="180" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C180" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="181" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="181" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C181" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="183" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="183" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C183" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="184" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="184" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C184" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="186" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="186" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C186" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="187" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="187" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C187" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="189" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="189" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C189" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="190" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="190" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C190" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="192" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="192" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C192" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="193" spans="3:3" x14ac:dyDescent="0.35">
+    <row r="193" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C193" t="s">
         <v>259</v>
       </c>
@@ -4056,1138 +4225,1138 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E778048-4A4A-4355-AB90-ACBFEF73D348}">
   <dimension ref="A1:AC131"/>
-  <sheetFormatPr defaultColWidth="2.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="5"/>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="5"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B33" s="5" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B34" s="5"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B35" s="5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B36" s="6" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B37" s="6"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B38" s="6" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B39" s="6"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B40" s="6" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>278</v>
       </c>
       <c r="B42" s="6"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B43" s="3"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B44" s="12" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B47" s="3"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B48" s="12" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="51" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B51" s="3"/>
     </row>
-    <row r="52" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="27" t="s">
+    <row r="52" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="C52" s="27" t="s">
+      <c r="C52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="D52" s="27" t="s">
+      <c r="D52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="E52" s="27" t="s">
+      <c r="E52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="F52" s="27" t="s">
+      <c r="F52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="G52" s="27" t="s">
+      <c r="G52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="H52" s="27" t="s">
+      <c r="H52" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="I52" s="27" t="s">
+      <c r="I52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="J52" s="27" t="s">
+      <c r="J52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="K52" s="27" t="s">
+      <c r="K52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="L52" s="27" t="s">
+      <c r="L52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="M52" s="27" t="s">
+      <c r="M52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="N52" s="27" t="s">
+      <c r="N52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="O52" s="27" t="s">
+      <c r="O52" s="30" t="s">
         <v>279</v>
       </c>
-      <c r="P52" s="27" t="s">
+      <c r="P52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="Q52" s="27" t="s">
+      <c r="Q52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="R52" s="27" t="s">
+      <c r="R52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="S52" s="27" t="s">
+      <c r="S52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="T52" s="27" t="s">
+      <c r="T52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="U52" s="27" t="s">
+      <c r="U52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="V52" s="27" t="s">
+      <c r="V52" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="W52" s="27" t="s">
+      <c r="W52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="X52" s="27" t="s">
+      <c r="X52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="Y52" s="27" t="s">
+      <c r="Y52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="Z52" s="27" t="s">
+      <c r="Z52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="AA52" s="27" t="s">
+      <c r="AA52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="AB52" s="27" t="s">
+      <c r="AB52" s="30" t="s">
         <v>284</v>
       </c>
-      <c r="AC52" s="27" t="s">
+      <c r="AC52" s="30" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="53" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B53" s="26" t="s">
+    <row r="53" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="C53" s="26" t="s">
+      <c r="C53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="D53" s="26" t="s">
+      <c r="D53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="E53" s="26" t="s">
+      <c r="E53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="F53" s="26" t="s">
+      <c r="F53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="G53" s="26" t="s">
+      <c r="G53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="H53" s="26" t="s">
+      <c r="H53" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="I53" s="26" t="s">
+      <c r="I53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="J53" s="26" t="s">
+      <c r="J53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="K53" s="26" t="s">
+      <c r="K53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="L53" s="26" t="s">
+      <c r="L53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="M53" s="26" t="s">
+      <c r="M53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="N53" s="26" t="s">
+      <c r="N53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="O53" s="26" t="s">
+      <c r="O53" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="P53" s="26" t="s">
+      <c r="P53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="Q53" s="26" t="s">
+      <c r="Q53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="R53" s="26" t="s">
+      <c r="R53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="S53" s="26" t="s">
+      <c r="S53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="T53" s="26" t="s">
+      <c r="T53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="U53" s="26" t="s">
+      <c r="U53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="V53" s="26" t="s">
+      <c r="V53" s="29" t="s">
         <v>286</v>
       </c>
-      <c r="W53" s="26" t="s">
+      <c r="W53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="X53" s="26" t="s">
+      <c r="X53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="Y53" s="26" t="s">
+      <c r="Y53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="Z53" s="26" t="s">
+      <c r="Z53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="AA53" s="26" t="s">
+      <c r="AA53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="AB53" s="26" t="s">
+      <c r="AB53" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="AC53" s="26" t="s">
+      <c r="AC53" s="29" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="54" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B54" s="26" t="s">
+    <row r="54" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="C54" s="26" t="s">
+      <c r="C54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="D54" s="26" t="s">
+      <c r="D54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="E54" s="26" t="s">
+      <c r="E54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="F54" s="26" t="s">
+      <c r="F54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="G54" s="26" t="s">
+      <c r="G54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="H54" s="26" t="s">
+      <c r="H54" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="I54" s="26" t="s">
+      <c r="I54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="J54" s="26" t="s">
+      <c r="J54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="K54" s="26" t="s">
+      <c r="K54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="L54" s="26" t="s">
+      <c r="L54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="M54" s="26" t="s">
+      <c r="M54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="N54" s="26" t="s">
+      <c r="N54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="O54" s="26" t="s">
+      <c r="O54" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="P54" s="26" t="s">
+      <c r="P54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="Q54" s="26" t="s">
+      <c r="Q54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="R54" s="26" t="s">
+      <c r="R54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="S54" s="26" t="s">
+      <c r="S54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="T54" s="26" t="s">
+      <c r="T54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="U54" s="26" t="s">
+      <c r="U54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="V54" s="26" t="s">
+      <c r="V54" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="W54" s="26" t="s">
+      <c r="W54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="X54" s="26" t="s">
+      <c r="X54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="Y54" s="26" t="s">
+      <c r="Y54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="Z54" s="26" t="s">
+      <c r="Z54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="AA54" s="26" t="s">
+      <c r="AA54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="AB54" s="26" t="s">
+      <c r="AB54" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="AC54" s="26" t="s">
+      <c r="AC54" s="29" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="55" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B55" s="26" t="s">
+    <row r="55" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="C55" s="26" t="s">
+      <c r="C55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="D55" s="26" t="s">
+      <c r="D55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="E55" s="26" t="s">
+      <c r="E55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="F55" s="26" t="s">
+      <c r="F55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="G55" s="26" t="s">
+      <c r="G55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="H55" s="26" t="s">
+      <c r="H55" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="I55" s="26" t="s">
+      <c r="I55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="J55" s="26" t="s">
+      <c r="J55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="K55" s="26" t="s">
+      <c r="K55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="L55" s="26" t="s">
+      <c r="L55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="M55" s="26" t="s">
+      <c r="M55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="N55" s="26" t="s">
+      <c r="N55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="O55" s="26" t="s">
+      <c r="O55" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="P55" s="26" t="s">
+      <c r="P55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="Q55" s="26" t="s">
+      <c r="Q55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="R55" s="26" t="s">
+      <c r="R55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="S55" s="26" t="s">
+      <c r="S55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="T55" s="26" t="s">
+      <c r="T55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="U55" s="26" t="s">
+      <c r="U55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="V55" s="26" t="s">
+      <c r="V55" s="29" t="s">
         <v>294</v>
       </c>
-      <c r="W55" s="26" t="s">
+      <c r="W55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="X55" s="26" t="s">
+      <c r="X55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="Y55" s="26" t="s">
+      <c r="Y55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="Z55" s="26" t="s">
+      <c r="Z55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="AA55" s="26" t="s">
+      <c r="AA55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="AB55" s="26" t="s">
+      <c r="AB55" s="29" t="s">
         <v>295</v>
       </c>
-      <c r="AC55" s="26" t="s">
+      <c r="AC55" s="29" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="56" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B56" s="26" t="s">
+    <row r="56" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="C56" s="26" t="s">
+      <c r="C56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="D56" s="26" t="s">
+      <c r="D56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="E56" s="26" t="s">
+      <c r="E56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="F56" s="26" t="s">
+      <c r="F56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="G56" s="26" t="s">
+      <c r="G56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="H56" s="26" t="s">
+      <c r="H56" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="I56" s="26" t="s">
+      <c r="I56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="J56" s="26" t="s">
+      <c r="J56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="K56" s="26" t="s">
+      <c r="K56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="L56" s="26" t="s">
+      <c r="L56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="M56" s="26" t="s">
+      <c r="M56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="N56" s="26" t="s">
+      <c r="N56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="O56" s="26" t="s">
+      <c r="O56" s="29" t="s">
         <v>297</v>
       </c>
-      <c r="P56" s="26" t="s">
+      <c r="P56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="Q56" s="26" t="s">
+      <c r="Q56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="R56" s="26" t="s">
+      <c r="R56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="S56" s="26" t="s">
+      <c r="S56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="T56" s="26" t="s">
+      <c r="T56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="U56" s="26" t="s">
+      <c r="U56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="V56" s="26" t="s">
+      <c r="V56" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="W56" s="26" t="s">
+      <c r="W56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="X56" s="26" t="s">
+      <c r="X56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="Y56" s="26" t="s">
+      <c r="Y56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="Z56" s="26" t="s">
+      <c r="Z56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="AA56" s="26" t="s">
+      <c r="AA56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="AB56" s="26" t="s">
+      <c r="AB56" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="AC56" s="26" t="s">
+      <c r="AC56" s="29" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="57" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B57" s="26" t="s">
+    <row r="57" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="C57" s="26" t="s">
+      <c r="C57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="D57" s="26" t="s">
+      <c r="D57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="E57" s="26" t="s">
+      <c r="E57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="F57" s="26" t="s">
+      <c r="F57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="26" t="s">
+      <c r="G57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="H57" s="26" t="s">
+      <c r="H57" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="I57" s="26" t="s">
+      <c r="I57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="J57" s="26" t="s">
+      <c r="J57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="K57" s="26" t="s">
+      <c r="K57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="L57" s="26" t="s">
+      <c r="L57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="M57" s="26" t="s">
+      <c r="M57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="N57" s="26" t="s">
+      <c r="N57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="O57" s="26" t="s">
+      <c r="O57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="P57" s="26" t="s">
+      <c r="P57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="Q57" s="26" t="s">
+      <c r="Q57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="R57" s="26" t="s">
+      <c r="R57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="S57" s="26" t="s">
+      <c r="S57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="T57" s="26" t="s">
+      <c r="T57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="U57" s="26" t="s">
+      <c r="U57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="V57" s="26" t="s">
+      <c r="V57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="W57" s="26" t="s">
+      <c r="W57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="X57" s="26" t="s">
+      <c r="X57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="Y57" s="26" t="s">
+      <c r="Y57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="Z57" s="26" t="s">
+      <c r="Z57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="AA57" s="26" t="s">
+      <c r="AA57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="AB57" s="26" t="s">
+      <c r="AB57" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="AC57" s="26" t="s">
+      <c r="AC57" s="29" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="58" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B58" s="26" t="s">
+    <row r="58" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="C58" s="26" t="s">
+      <c r="C58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="D58" s="26" t="s">
+      <c r="D58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="E58" s="26" t="s">
+      <c r="E58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="F58" s="26" t="s">
+      <c r="F58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="G58" s="26" t="s">
+      <c r="G58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="H58" s="26" t="s">
+      <c r="H58" s="29" t="s">
         <v>303</v>
       </c>
-      <c r="I58" s="26" t="s">
+      <c r="I58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="J58" s="26" t="s">
+      <c r="J58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="K58" s="26" t="s">
+      <c r="K58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="L58" s="26" t="s">
+      <c r="L58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="M58" s="26" t="s">
+      <c r="M58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="N58" s="26" t="s">
+      <c r="N58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="O58" s="26" t="s">
+      <c r="O58" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="P58" s="26" t="s">
+      <c r="P58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="Q58" s="26" t="s">
+      <c r="Q58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="R58" s="26" t="s">
+      <c r="R58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="S58" s="26" t="s">
+      <c r="S58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="T58" s="26" t="s">
+      <c r="T58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="U58" s="26" t="s">
+      <c r="U58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="V58" s="26" t="s">
+      <c r="V58" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="W58" s="26" t="s">
+      <c r="W58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="X58" s="26" t="s">
+      <c r="X58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="Y58" s="26" t="s">
+      <c r="Y58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="Z58" s="26" t="s">
+      <c r="Z58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="AA58" s="26" t="s">
+      <c r="AA58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="AB58" s="26" t="s">
+      <c r="AB58" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="AC58" s="26" t="s">
+      <c r="AC58" s="29" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="59" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B59" s="26" t="s">
+    <row r="59" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="C59" s="26" t="s">
+      <c r="C59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="D59" s="26" t="s">
+      <c r="D59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="E59" s="26" t="s">
+      <c r="E59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="F59" s="26" t="s">
+      <c r="F59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="G59" s="26" t="s">
+      <c r="G59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="H59" s="26" t="s">
+      <c r="H59" s="29" t="s">
         <v>307</v>
       </c>
-      <c r="I59" s="26" t="s">
+      <c r="I59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="J59" s="26" t="s">
+      <c r="J59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="K59" s="26" t="s">
+      <c r="K59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="L59" s="26" t="s">
+      <c r="L59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="M59" s="26" t="s">
+      <c r="M59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="N59" s="26" t="s">
+      <c r="N59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="O59" s="26" t="s">
+      <c r="O59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="P59" s="26" t="s">
+      <c r="P59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="Q59" s="26" t="s">
+      <c r="Q59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="R59" s="26" t="s">
+      <c r="R59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="S59" s="26" t="s">
+      <c r="S59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="T59" s="26" t="s">
+      <c r="T59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="U59" s="26" t="s">
+      <c r="U59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="V59" s="26" t="s">
+      <c r="V59" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="W59" s="26" t="s">
+      <c r="W59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="X59" s="26" t="s">
+      <c r="X59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="Y59" s="26" t="s">
+      <c r="Y59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="Z59" s="26" t="s">
+      <c r="Z59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="AA59" s="26" t="s">
+      <c r="AA59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="AB59" s="26" t="s">
+      <c r="AB59" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="AC59" s="26" t="s">
+      <c r="AC59" s="29" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="62" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="64" spans="1:29" x14ac:dyDescent="0.35">
-      <c r="B64" s="16" t="s">
+    <row r="64" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B64" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="16"/>
-      <c r="G64" s="16"/>
-      <c r="H64" s="16" t="s">
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="20"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-      <c r="K64" s="16"/>
-      <c r="L64" s="16"/>
-      <c r="M64" s="16"/>
-    </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B65" s="16" t="s">
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
+      <c r="K64" s="20"/>
+      <c r="L64" s="20"/>
+      <c r="M64" s="20"/>
+    </row>
+    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B65" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="16"/>
-      <c r="E65" s="16"/>
-      <c r="F65" s="16"/>
-      <c r="G65" s="16"/>
-      <c r="H65" s="16" t="s">
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="20"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="20" t="s">
         <v>316</v>
       </c>
-      <c r="I65" s="16"/>
-      <c r="J65" s="16"/>
-      <c r="K65" s="16"/>
-      <c r="L65" s="16"/>
-      <c r="M65" s="16"/>
-    </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B66" s="16" t="s">
+      <c r="I65" s="20"/>
+      <c r="J65" s="20"/>
+      <c r="K65" s="20"/>
+      <c r="L65" s="20"/>
+      <c r="M65" s="20"/>
+    </row>
+    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B66" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="C66" s="16"/>
-      <c r="D66" s="16"/>
-      <c r="E66" s="16"/>
-      <c r="F66" s="16"/>
-      <c r="G66" s="16"/>
-      <c r="H66" s="16" t="s">
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20" t="s">
         <v>317</v>
       </c>
-      <c r="I66" s="16"/>
-      <c r="J66" s="16"/>
-      <c r="K66" s="16"/>
-      <c r="L66" s="16"/>
-      <c r="M66" s="16"/>
-    </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B67" s="16" t="s">
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+      <c r="M66" s="20"/>
+    </row>
+    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B67" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="C67" s="16"/>
-      <c r="D67" s="16"/>
-      <c r="E67" s="16"/>
-      <c r="F67" s="16"/>
-      <c r="G67" s="16"/>
-      <c r="H67" s="16" t="s">
+      <c r="C67" s="20"/>
+      <c r="D67" s="20"/>
+      <c r="E67" s="20"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="20" t="s">
         <v>313</v>
       </c>
-      <c r="I67" s="16"/>
-      <c r="J67" s="16"/>
-      <c r="K67" s="16"/>
-      <c r="L67" s="16"/>
-      <c r="M67" s="16"/>
-    </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B68" s="16" t="s">
+      <c r="I67" s="20"/>
+      <c r="J67" s="20"/>
+      <c r="K67" s="20"/>
+      <c r="L67" s="20"/>
+      <c r="M67" s="20"/>
+    </row>
+    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B68" s="20" t="s">
         <v>300</v>
       </c>
-      <c r="C68" s="16"/>
-      <c r="D68" s="16"/>
-      <c r="E68" s="16"/>
-      <c r="F68" s="16"/>
-      <c r="G68" s="16"/>
-      <c r="H68" s="16" t="s">
+      <c r="C68" s="20"/>
+      <c r="D68" s="20"/>
+      <c r="E68" s="20"/>
+      <c r="F68" s="20"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="20" t="s">
         <v>312</v>
       </c>
-      <c r="I68" s="16"/>
-      <c r="J68" s="16"/>
-      <c r="K68" s="16"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="16"/>
-    </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B69" s="16" t="s">
+      <c r="I68" s="20"/>
+      <c r="J68" s="20"/>
+      <c r="K68" s="20"/>
+      <c r="L68" s="20"/>
+      <c r="M68" s="20"/>
+    </row>
+    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B69" s="20" t="s">
         <v>303</v>
       </c>
-      <c r="C69" s="16"/>
-      <c r="D69" s="16"/>
-      <c r="E69" s="16"/>
-      <c r="F69" s="16"/>
-      <c r="G69" s="16"/>
-      <c r="H69" s="16" t="s">
+      <c r="C69" s="20"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="I69" s="16"/>
-      <c r="J69" s="16"/>
-      <c r="K69" s="16"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="16"/>
-    </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B70" s="16" t="s">
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+      <c r="L69" s="20"/>
+      <c r="M69" s="20"/>
+    </row>
+    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B70" s="20" t="s">
         <v>307</v>
       </c>
-      <c r="C70" s="16"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="16"/>
-      <c r="F70" s="16"/>
-      <c r="G70" s="16"/>
-      <c r="H70" s="16" t="s">
+      <c r="C70" s="20"/>
+      <c r="D70" s="20"/>
+      <c r="E70" s="20"/>
+      <c r="F70" s="20"/>
+      <c r="G70" s="20"/>
+      <c r="H70" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-    </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="I70" s="20"/>
+      <c r="J70" s="20"/>
+      <c r="K70" s="20"/>
+      <c r="L70" s="20"/>
+      <c r="M70" s="20"/>
+    </row>
+    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="7" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="7" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B77" s="7"/>
     </row>
-    <row r="98" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B98" s="13"/>
-      <c r="C98" s="13"/>
-      <c r="D98" s="13"/>
-      <c r="E98" s="13"/>
-      <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
-      <c r="H98" s="13"/>
-      <c r="I98" s="13"/>
-      <c r="J98" s="13"/>
-      <c r="K98" s="13"/>
-      <c r="L98" s="13"/>
-      <c r="M98" s="13"/>
-    </row>
-    <row r="99" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B99" s="13"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="13"/>
-      <c r="E99" s="13"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="13"/>
-      <c r="I99" s="13"/>
-      <c r="J99" s="13"/>
-      <c r="K99" s="13"/>
-      <c r="L99" s="13"/>
-      <c r="M99" s="13"/>
-    </row>
-    <row r="100" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B100" s="13"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="13"/>
-      <c r="E100" s="13"/>
-      <c r="F100" s="13"/>
-      <c r="G100" s="13"/>
-      <c r="H100" s="13"/>
-      <c r="I100" s="13"/>
-      <c r="J100" s="13"/>
-      <c r="K100" s="13"/>
-      <c r="L100" s="13"/>
-      <c r="M100" s="13"/>
-    </row>
-    <row r="101" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B101" s="13"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="13"/>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="13"/>
-      <c r="I101" s="13"/>
-      <c r="J101" s="13"/>
-      <c r="K101" s="13"/>
-      <c r="L101" s="13"/>
-      <c r="M101" s="13"/>
-    </row>
-    <row r="102" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B102" s="13"/>
-      <c r="C102" s="13"/>
-      <c r="D102" s="13"/>
-      <c r="E102" s="13"/>
-      <c r="F102" s="13"/>
-      <c r="G102" s="13"/>
-      <c r="H102" s="13"/>
-      <c r="I102" s="13"/>
-      <c r="J102" s="13"/>
-      <c r="K102" s="13"/>
-      <c r="L102" s="13"/>
-      <c r="M102" s="13"/>
-    </row>
-    <row r="103" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B103" s="13"/>
-      <c r="C103" s="13"/>
-      <c r="D103" s="13"/>
-      <c r="E103" s="13"/>
-      <c r="F103" s="13"/>
-      <c r="G103" s="13"/>
-      <c r="H103" s="13"/>
-      <c r="I103" s="13"/>
-      <c r="J103" s="13"/>
-      <c r="K103" s="13"/>
-      <c r="L103" s="13"/>
-      <c r="M103" s="13"/>
-    </row>
-    <row r="104" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B104" s="13"/>
-      <c r="C104" s="13"/>
-      <c r="D104" s="13"/>
-      <c r="E104" s="13"/>
-      <c r="F104" s="13"/>
-      <c r="G104" s="13"/>
-      <c r="H104" s="13"/>
-      <c r="I104" s="13"/>
-      <c r="J104" s="13"/>
-      <c r="K104" s="13"/>
-      <c r="L104" s="13"/>
-      <c r="M104" s="13"/>
-    </row>
-    <row r="105" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B105" s="13"/>
-      <c r="C105" s="13"/>
-      <c r="D105" s="13"/>
-      <c r="E105" s="13"/>
-      <c r="F105" s="13"/>
-      <c r="G105" s="13"/>
-      <c r="H105" s="13"/>
-      <c r="I105" s="13"/>
-      <c r="J105" s="13"/>
-      <c r="K105" s="13"/>
-      <c r="L105" s="13"/>
-      <c r="M105" s="13"/>
-    </row>
-    <row r="106" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B106" s="13"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="13"/>
-      <c r="E106" s="13"/>
-      <c r="F106" s="13"/>
-      <c r="G106" s="13"/>
-      <c r="H106" s="13"/>
-      <c r="I106" s="13"/>
-      <c r="J106" s="13"/>
-      <c r="K106" s="13"/>
-      <c r="L106" s="13"/>
-      <c r="M106" s="13"/>
-    </row>
-    <row r="107" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B107" s="13"/>
-      <c r="C107" s="13"/>
-      <c r="D107" s="13"/>
-      <c r="E107" s="13"/>
-      <c r="F107" s="13"/>
-      <c r="G107" s="13"/>
-      <c r="H107" s="13"/>
-      <c r="I107" s="13"/>
-      <c r="J107" s="13"/>
-      <c r="K107" s="13"/>
-      <c r="L107" s="13"/>
-      <c r="M107" s="13"/>
-    </row>
-    <row r="129" spans="13:13" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B98" s="17"/>
+      <c r="C98" s="17"/>
+      <c r="D98" s="17"/>
+      <c r="E98" s="17"/>
+      <c r="F98" s="17"/>
+      <c r="G98" s="17"/>
+      <c r="H98" s="17"/>
+      <c r="I98" s="17"/>
+      <c r="J98" s="17"/>
+      <c r="K98" s="17"/>
+      <c r="L98" s="17"/>
+      <c r="M98" s="17"/>
+    </row>
+    <row r="99" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B99" s="17"/>
+      <c r="C99" s="17"/>
+      <c r="D99" s="17"/>
+      <c r="E99" s="17"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
+      <c r="H99" s="17"/>
+      <c r="I99" s="17"/>
+      <c r="J99" s="17"/>
+      <c r="K99" s="17"/>
+      <c r="L99" s="17"/>
+      <c r="M99" s="17"/>
+    </row>
+    <row r="100" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B100" s="17"/>
+      <c r="C100" s="17"/>
+      <c r="D100" s="17"/>
+      <c r="E100" s="17"/>
+      <c r="F100" s="17"/>
+      <c r="G100" s="17"/>
+      <c r="H100" s="17"/>
+      <c r="I100" s="17"/>
+      <c r="J100" s="17"/>
+      <c r="K100" s="17"/>
+      <c r="L100" s="17"/>
+      <c r="M100" s="17"/>
+    </row>
+    <row r="101" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B101" s="17"/>
+      <c r="C101" s="17"/>
+      <c r="D101" s="17"/>
+      <c r="E101" s="17"/>
+      <c r="F101" s="17"/>
+      <c r="G101" s="17"/>
+      <c r="H101" s="17"/>
+      <c r="I101" s="17"/>
+      <c r="J101" s="17"/>
+      <c r="K101" s="17"/>
+      <c r="L101" s="17"/>
+      <c r="M101" s="17"/>
+    </row>
+    <row r="102" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B102" s="17"/>
+      <c r="C102" s="17"/>
+      <c r="D102" s="17"/>
+      <c r="E102" s="17"/>
+      <c r="F102" s="17"/>
+      <c r="G102" s="17"/>
+      <c r="H102" s="17"/>
+      <c r="I102" s="17"/>
+      <c r="J102" s="17"/>
+      <c r="K102" s="17"/>
+      <c r="L102" s="17"/>
+      <c r="M102" s="17"/>
+    </row>
+    <row r="103" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B103" s="17"/>
+      <c r="C103" s="17"/>
+      <c r="D103" s="17"/>
+      <c r="E103" s="17"/>
+      <c r="F103" s="17"/>
+      <c r="G103" s="17"/>
+      <c r="H103" s="17"/>
+      <c r="I103" s="17"/>
+      <c r="J103" s="17"/>
+      <c r="K103" s="17"/>
+      <c r="L103" s="17"/>
+      <c r="M103" s="17"/>
+    </row>
+    <row r="104" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B104" s="17"/>
+      <c r="C104" s="17"/>
+      <c r="D104" s="17"/>
+      <c r="E104" s="17"/>
+      <c r="F104" s="17"/>
+      <c r="G104" s="17"/>
+      <c r="H104" s="17"/>
+      <c r="I104" s="17"/>
+      <c r="J104" s="17"/>
+      <c r="K104" s="17"/>
+      <c r="L104" s="17"/>
+      <c r="M104" s="17"/>
+    </row>
+    <row r="105" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B105" s="17"/>
+      <c r="C105" s="17"/>
+      <c r="D105" s="17"/>
+      <c r="E105" s="17"/>
+      <c r="F105" s="17"/>
+      <c r="G105" s="17"/>
+      <c r="H105" s="17"/>
+      <c r="I105" s="17"/>
+      <c r="J105" s="17"/>
+      <c r="K105" s="17"/>
+      <c r="L105" s="17"/>
+      <c r="M105" s="17"/>
+    </row>
+    <row r="106" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B106" s="17"/>
+      <c r="C106" s="17"/>
+      <c r="D106" s="17"/>
+      <c r="E106" s="17"/>
+      <c r="F106" s="17"/>
+      <c r="G106" s="17"/>
+      <c r="H106" s="17"/>
+      <c r="I106" s="17"/>
+      <c r="J106" s="17"/>
+      <c r="K106" s="17"/>
+      <c r="L106" s="17"/>
+      <c r="M106" s="17"/>
+    </row>
+    <row r="107" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B107" s="17"/>
+      <c r="C107" s="17"/>
+      <c r="D107" s="17"/>
+      <c r="E107" s="17"/>
+      <c r="F107" s="17"/>
+      <c r="G107" s="17"/>
+      <c r="H107" s="17"/>
+      <c r="I107" s="17"/>
+      <c r="J107" s="17"/>
+      <c r="K107" s="17"/>
+      <c r="L107" s="17"/>
+      <c r="M107" s="17"/>
+    </row>
+    <row r="129" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M129" s="7"/>
     </row>
-    <row r="131" spans="13:13" x14ac:dyDescent="0.35">
+    <row r="131" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M131" s="7"/>
     </row>
   </sheetData>
@@ -5266,290 +5435,592 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B495B359-6014-42AA-8F6E-00A02E8709AE}">
+  <dimension ref="A1:M88"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.85546875" style="10"/>
+    <col min="2" max="2" width="21.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="25" style="10" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" style="10" customWidth="1"/>
+    <col min="6" max="16384" width="2.85546875" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="10" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="10" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="10" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="10" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="10" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="10" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="10" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="10" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="10" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="9" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="9" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="10" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>335</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="10" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="9" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="10" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
+      <c r="K55" s="16"/>
+      <c r="L55" s="16"/>
+      <c r="M55" s="16"/>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
+      <c r="H56" s="16"/>
+      <c r="I56" s="16"/>
+      <c r="J56" s="16"/>
+      <c r="K56" s="16"/>
+      <c r="L56" s="16"/>
+      <c r="M56" s="16"/>
+    </row>
+    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
+      <c r="J57" s="16"/>
+      <c r="K57" s="16"/>
+      <c r="L57" s="16"/>
+      <c r="M57" s="16"/>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
+      <c r="J58" s="16"/>
+      <c r="K58" s="16"/>
+      <c r="L58" s="16"/>
+      <c r="M58" s="16"/>
+    </row>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
+      <c r="J59" s="16"/>
+      <c r="K59" s="16"/>
+      <c r="L59" s="16"/>
+      <c r="M59" s="16"/>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="16"/>
+      <c r="I60" s="16"/>
+      <c r="J60" s="16"/>
+      <c r="K60" s="16"/>
+      <c r="L60" s="16"/>
+      <c r="M60" s="16"/>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B61" s="16"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="16"/>
+      <c r="I61" s="16"/>
+      <c r="J61" s="16"/>
+      <c r="K61" s="16"/>
+      <c r="L61" s="16"/>
+      <c r="M61" s="16"/>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B62" s="16"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="16"/>
+      <c r="I62" s="16"/>
+      <c r="J62" s="16"/>
+      <c r="K62" s="16"/>
+      <c r="L62" s="16"/>
+      <c r="M62" s="16"/>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16"/>
+      <c r="J63" s="16"/>
+      <c r="K63" s="16"/>
+      <c r="L63" s="16"/>
+      <c r="M63" s="16"/>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
+      <c r="J64" s="16"/>
+      <c r="K64" s="16"/>
+      <c r="L64" s="16"/>
+      <c r="M64" s="16"/>
+    </row>
+    <row r="86" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M86" s="9"/>
+    </row>
+    <row r="88" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M88" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B55:G55"/>
+    <mergeCell ref="H55:M55"/>
+    <mergeCell ref="B56:G56"/>
+    <mergeCell ref="H56:M56"/>
+    <mergeCell ref="B57:G57"/>
+    <mergeCell ref="H57:M57"/>
+    <mergeCell ref="B58:G58"/>
+    <mergeCell ref="H58:M58"/>
+    <mergeCell ref="B59:G59"/>
+    <mergeCell ref="H59:M59"/>
+    <mergeCell ref="B60:G60"/>
+    <mergeCell ref="H60:M60"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="H64:M64"/>
+    <mergeCell ref="B61:G61"/>
+    <mergeCell ref="H61:M61"/>
+    <mergeCell ref="B62:G62"/>
+    <mergeCell ref="H62:M62"/>
+    <mergeCell ref="B63:G63"/>
+    <mergeCell ref="H63:M63"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5119FBB-A220-4E1A-9A2A-E6AE56D555F6}">
-  <dimension ref="A1:M153"/>
-  <sheetFormatPr defaultColWidth="2.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B28:M153"/>
+  <sheetFormatPr defaultColWidth="2.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="2.85546875" style="10"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1"/>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B25" s="5"/>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B27" s="6"/>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B28" s="3"/>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B29" s="5"/>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B30" s="2"/>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B31" s="6"/>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B32" s="3"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B33" s="5"/>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B34" s="2"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B35" s="6"/>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B36" s="3"/>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B37" s="5"/>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B38" s="2"/>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B39" s="6"/>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B40" s="3"/>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B42" s="4"/>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B43" s="5"/>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B44" s="2"/>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B45" s="6"/>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B46" s="3"/>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B47" s="5"/>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B48" s="2"/>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B49" s="6"/>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B50" s="3"/>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B51" s="5"/>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B52" s="2"/>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B53" s="6"/>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B54" s="3"/>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B55" s="5"/>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B56" s="2"/>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B57" s="6"/>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B58" s="3"/>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B60" s="4"/>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B61" s="5"/>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B62" s="2"/>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B63" s="6"/>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B64" s="3"/>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B65" s="5"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B66" s="2"/>
-    </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B67" s="6"/>
-    </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B68" s="3"/>
-    </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B99" s="7"/>
-    </row>
-    <row r="120" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B120" s="13"/>
-      <c r="C120" s="13"/>
-      <c r="D120" s="13"/>
-      <c r="E120" s="13"/>
-      <c r="F120" s="13"/>
-      <c r="G120" s="13"/>
-      <c r="H120" s="13"/>
-      <c r="I120" s="13"/>
-      <c r="J120" s="13"/>
-      <c r="K120" s="13"/>
-      <c r="L120" s="13"/>
-      <c r="M120" s="13"/>
-    </row>
-    <row r="121" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B121" s="13"/>
-      <c r="C121" s="13"/>
-      <c r="D121" s="13"/>
-      <c r="E121" s="13"/>
-      <c r="F121" s="13"/>
-      <c r="G121" s="13"/>
-      <c r="H121" s="13"/>
-      <c r="I121" s="13"/>
-      <c r="J121" s="13"/>
-      <c r="K121" s="13"/>
-      <c r="L121" s="13"/>
-      <c r="M121" s="13"/>
-    </row>
-    <row r="122" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B122" s="13"/>
-      <c r="C122" s="13"/>
-      <c r="D122" s="13"/>
-      <c r="E122" s="13"/>
-      <c r="F122" s="13"/>
-      <c r="G122" s="13"/>
-      <c r="H122" s="13"/>
-      <c r="I122" s="13"/>
-      <c r="J122" s="13"/>
-      <c r="K122" s="13"/>
-      <c r="L122" s="13"/>
-      <c r="M122" s="13"/>
-    </row>
-    <row r="123" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B123" s="13"/>
-      <c r="C123" s="13"/>
-      <c r="D123" s="13"/>
-      <c r="E123" s="13"/>
-      <c r="F123" s="13"/>
-      <c r="G123" s="13"/>
-      <c r="H123" s="13"/>
-      <c r="I123" s="13"/>
-      <c r="J123" s="13"/>
-      <c r="K123" s="13"/>
-      <c r="L123" s="13"/>
-      <c r="M123" s="13"/>
-    </row>
-    <row r="124" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B124" s="13"/>
-      <c r="C124" s="13"/>
-      <c r="D124" s="13"/>
-      <c r="E124" s="13"/>
-      <c r="F124" s="13"/>
-      <c r="G124" s="13"/>
-      <c r="H124" s="13"/>
-      <c r="I124" s="13"/>
-      <c r="J124" s="13"/>
-      <c r="K124" s="13"/>
-      <c r="L124" s="13"/>
-      <c r="M124" s="13"/>
-    </row>
-    <row r="125" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B125" s="13"/>
-      <c r="C125" s="13"/>
-      <c r="D125" s="13"/>
-      <c r="E125" s="13"/>
-      <c r="F125" s="13"/>
-      <c r="G125" s="13"/>
-      <c r="H125" s="13"/>
-      <c r="I125" s="13"/>
-      <c r="J125" s="13"/>
-      <c r="K125" s="13"/>
-      <c r="L125" s="13"/>
-      <c r="M125" s="13"/>
-    </row>
-    <row r="126" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B126" s="13"/>
-      <c r="C126" s="13"/>
-      <c r="D126" s="13"/>
-      <c r="E126" s="13"/>
-      <c r="F126" s="13"/>
-      <c r="G126" s="13"/>
-      <c r="H126" s="13"/>
-      <c r="I126" s="13"/>
-      <c r="J126" s="13"/>
-      <c r="K126" s="13"/>
-      <c r="L126" s="13"/>
-      <c r="M126" s="13"/>
-    </row>
-    <row r="127" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B127" s="13"/>
-      <c r="C127" s="13"/>
-      <c r="D127" s="13"/>
-      <c r="E127" s="13"/>
-      <c r="F127" s="13"/>
-      <c r="G127" s="13"/>
-      <c r="H127" s="13"/>
-      <c r="I127" s="13"/>
-      <c r="J127" s="13"/>
-      <c r="K127" s="13"/>
-      <c r="L127" s="13"/>
-      <c r="M127" s="13"/>
-    </row>
-    <row r="128" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B128" s="13"/>
-      <c r="C128" s="13"/>
-      <c r="D128" s="13"/>
-      <c r="E128" s="13"/>
-      <c r="F128" s="13"/>
-      <c r="G128" s="13"/>
-      <c r="H128" s="13"/>
-      <c r="I128" s="13"/>
-      <c r="J128" s="13"/>
-      <c r="K128" s="13"/>
-      <c r="L128" s="13"/>
-      <c r="M128" s="13"/>
-    </row>
-    <row r="129" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B129" s="13"/>
-      <c r="C129" s="13"/>
-      <c r="D129" s="13"/>
-      <c r="E129" s="13"/>
-      <c r="F129" s="13"/>
-      <c r="G129" s="13"/>
-      <c r="H129" s="13"/>
-      <c r="I129" s="13"/>
-      <c r="J129" s="13"/>
-      <c r="K129" s="13"/>
-      <c r="L129" s="13"/>
-      <c r="M129" s="13"/>
-    </row>
-    <row r="151" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M151" s="7"/>
-    </row>
-    <row r="153" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M153" s="7"/>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="11"/>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="11"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="11"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="11"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46" s="11"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" s="11"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" s="11"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" s="11"/>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" s="11"/>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" s="11"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B99" s="9"/>
+    </row>
+    <row r="120" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B120" s="16"/>
+      <c r="C120" s="16"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="16"/>
+      <c r="F120" s="16"/>
+      <c r="G120" s="16"/>
+      <c r="H120" s="16"/>
+      <c r="I120" s="16"/>
+      <c r="J120" s="16"/>
+      <c r="K120" s="16"/>
+      <c r="L120" s="16"/>
+      <c r="M120" s="16"/>
+    </row>
+    <row r="121" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B121" s="16"/>
+      <c r="C121" s="16"/>
+      <c r="D121" s="16"/>
+      <c r="E121" s="16"/>
+      <c r="F121" s="16"/>
+      <c r="G121" s="16"/>
+      <c r="H121" s="16"/>
+      <c r="I121" s="16"/>
+      <c r="J121" s="16"/>
+      <c r="K121" s="16"/>
+      <c r="L121" s="16"/>
+      <c r="M121" s="16"/>
+    </row>
+    <row r="122" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B122" s="16"/>
+      <c r="C122" s="16"/>
+      <c r="D122" s="16"/>
+      <c r="E122" s="16"/>
+      <c r="F122" s="16"/>
+      <c r="G122" s="16"/>
+      <c r="H122" s="16"/>
+      <c r="I122" s="16"/>
+      <c r="J122" s="16"/>
+      <c r="K122" s="16"/>
+      <c r="L122" s="16"/>
+      <c r="M122" s="16"/>
+    </row>
+    <row r="123" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B123" s="16"/>
+      <c r="C123" s="16"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="16"/>
+      <c r="F123" s="16"/>
+      <c r="G123" s="16"/>
+      <c r="H123" s="16"/>
+      <c r="I123" s="16"/>
+      <c r="J123" s="16"/>
+      <c r="K123" s="16"/>
+      <c r="L123" s="16"/>
+      <c r="M123" s="16"/>
+    </row>
+    <row r="124" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B124" s="16"/>
+      <c r="C124" s="16"/>
+      <c r="D124" s="16"/>
+      <c r="E124" s="16"/>
+      <c r="F124" s="16"/>
+      <c r="G124" s="16"/>
+      <c r="H124" s="16"/>
+      <c r="I124" s="16"/>
+      <c r="J124" s="16"/>
+      <c r="K124" s="16"/>
+      <c r="L124" s="16"/>
+      <c r="M124" s="16"/>
+    </row>
+    <row r="125" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B125" s="16"/>
+      <c r="C125" s="16"/>
+      <c r="D125" s="16"/>
+      <c r="E125" s="16"/>
+      <c r="F125" s="16"/>
+      <c r="G125" s="16"/>
+      <c r="H125" s="16"/>
+      <c r="I125" s="16"/>
+      <c r="J125" s="16"/>
+      <c r="K125" s="16"/>
+      <c r="L125" s="16"/>
+      <c r="M125" s="16"/>
+    </row>
+    <row r="126" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B126" s="16"/>
+      <c r="C126" s="16"/>
+      <c r="D126" s="16"/>
+      <c r="E126" s="16"/>
+      <c r="F126" s="16"/>
+      <c r="G126" s="16"/>
+      <c r="H126" s="16"/>
+      <c r="I126" s="16"/>
+      <c r="J126" s="16"/>
+      <c r="K126" s="16"/>
+      <c r="L126" s="16"/>
+      <c r="M126" s="16"/>
+    </row>
+    <row r="127" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B127" s="16"/>
+      <c r="C127" s="16"/>
+      <c r="D127" s="16"/>
+      <c r="E127" s="16"/>
+      <c r="F127" s="16"/>
+      <c r="G127" s="16"/>
+      <c r="H127" s="16"/>
+      <c r="I127" s="16"/>
+      <c r="J127" s="16"/>
+      <c r="K127" s="16"/>
+      <c r="L127" s="16"/>
+      <c r="M127" s="16"/>
+    </row>
+    <row r="128" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B128" s="16"/>
+      <c r="C128" s="16"/>
+      <c r="D128" s="16"/>
+      <c r="E128" s="16"/>
+      <c r="F128" s="16"/>
+      <c r="G128" s="16"/>
+      <c r="H128" s="16"/>
+      <c r="I128" s="16"/>
+      <c r="J128" s="16"/>
+      <c r="K128" s="16"/>
+      <c r="L128" s="16"/>
+      <c r="M128" s="16"/>
+    </row>
+    <row r="129" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B129" s="16"/>
+      <c r="C129" s="16"/>
+      <c r="D129" s="16"/>
+      <c r="E129" s="16"/>
+      <c r="F129" s="16"/>
+      <c r="G129" s="16"/>
+      <c r="H129" s="16"/>
+      <c r="I129" s="16"/>
+      <c r="J129" s="16"/>
+      <c r="K129" s="16"/>
+      <c r="L129" s="16"/>
+      <c r="M129" s="16"/>
+    </row>
+    <row r="151" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M151" s="9"/>
+    </row>
+    <row r="153" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M153" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="20">

</xml_diff>